<commit_message>
July month target added
</commit_message>
<xml_diff>
--- a/Target_fixed.xlsx
+++ b/Target_fixed.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ack\OneDrive\Documents\enforcement report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ack\My Drive\HINDUPUR-2022-2025\Target 2026-2027\Reports MVIs\web data files_github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689C5B1C-938E-4E3A-9D4F-FDBA22946508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF8D610-9E4F-44EC-AC2C-FD8B71F87450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14265" yWindow="4260" windowWidth="13350" windowHeight="11220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -537,6 +537,9 @@
       <c r="F2">
         <v>1138000</v>
       </c>
+      <c r="G2">
+        <v>1138000</v>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -557,6 +560,9 @@
       <c r="F3">
         <v>1138000</v>
       </c>
+      <c r="G3">
+        <v>1138000</v>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -577,6 +583,9 @@
       <c r="F4">
         <v>1138000</v>
       </c>
+      <c r="G4">
+        <v>1138000</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -597,6 +606,9 @@
       <c r="F5">
         <v>1138000</v>
       </c>
+      <c r="G5">
+        <v>1138000</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -617,6 +629,9 @@
       <c r="F6">
         <v>1138000</v>
       </c>
+      <c r="G6">
+        <v>1138000</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -635,6 +650,9 @@
         <v>1138000</v>
       </c>
       <c r="F7">
+        <v>1138000</v>
+      </c>
+      <c r="G7">
         <v>1138000</v>
       </c>
     </row>

</xml_diff>